<commit_message>
feat:change config Generate logic,add uijump test logic
</commit_message>
<xml_diff>
--- a/DesignData/Luban/Datas/UIJumpConfig.xlsx
+++ b/DesignData/Luban/Datas/UIJumpConfig.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
   <si>
     <t>##var</t>
   </si>
@@ -97,16 +97,40 @@
     <t>显式返回的跳转配置 ID</t>
   </si>
   <si>
-    <t>Luban 接入冒烟配置</t>
-  </si>
-  <si>
-    <t>LoadingUI</t>
+    <t>Open navigation home</t>
+  </si>
+  <si>
+    <t>NavigationHomeUI</t>
   </si>
   <si>
     <t>Overlay</t>
   </si>
   <si>
     <t>Disabled</t>
+  </si>
+  <si>
+    <t>Push detail and return home</t>
+  </si>
+  <si>
+    <t>NavigationDetailUI</t>
+  </si>
+  <si>
+    <t>Push</t>
+  </si>
+  <si>
+    <t>ReturnToSource</t>
+  </si>
+  <si>
+    <t>Overlay popup and return source</t>
+  </si>
+  <si>
+    <t>NavigationPopupUI</t>
+  </si>
+  <si>
+    <t>Overlay popup and skip detail</t>
+  </si>
+  <si>
+    <t>InheritSource</t>
   </si>
 </sst>
 </file>
@@ -1251,9 +1275,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="6"/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="6"/>
   <cols>
+    <col min="2" max="2" width="26.1111111111111" customWidth="1"/>
     <col min="3" max="3" width="45.5555555555556" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1287,7 +1312,6 @@
       <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2"/>
       <c r="D2" t="s">
         <v>9</v>
       </c>
@@ -1308,7 +1332,6 @@
       <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="C3"/>
       <c r="D3" t="s">
         <v>13</v>
       </c>
@@ -1347,7 +1370,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="B5">
-        <v>10001</v>
+        <v>1001</v>
       </c>
       <c r="C5" t="s">
         <v>21</v>
@@ -1362,6 +1385,66 @@
         <v>24</v>
       </c>
       <c r="G5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="B6">
+        <v>1002</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="B7">
+        <v>1003</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="B8">
+        <v>1004</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" t="s">
+        <v>32</v>
+      </c>
+      <c r="G8">
         <v>0</v>
       </c>
     </row>

</xml_diff>